<commit_message>
feat(codegen): add unique field accessors
</commit_message>
<xml_diff>
--- a/tests/testdata/excels/valid/Config.xlsx
+++ b/tests/testdata/excels/valid/Config.xlsx
@@ -1,95 +1,104 @@
 
 <file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
-  <si>
-    <t>*id</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+  <si>
+    <t>id#</t>
+  </si>
+  <si>
+    <t>name!</t>
+  </si>
+  <si>
+    <t>label*</t>
+  </si>
+  <si>
+    <t>enabled</t>
+  </si>
+  <si>
+    <t>score</t>
+  </si>
+  <si>
+    <t>big</t>
+  </si>
+  <si>
+    <t>ratio</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>createdAt</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>attrs</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>serverOnly</t>
+  </si>
+  <si>
+    <t>clientOnly!</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>int32</t>
+  </si>
+  <si>
+    <t>int64</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>double</t>
+  </si>
+  <si>
+    <t>datetime</t>
+  </si>
+  <si>
+    <t>array&lt;string&gt;</t>
+  </si>
+  <si>
+    <t>map&lt;string,int&gt;</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>client</t>
+  </si>
+  <si>
+    <t>server</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>srv</t>
+  </si>
+  <si>
+    <t>unique id</t>
   </si>
   <si>
     <t>name</t>
   </si>
   <si>
-    <t>enabled</t>
-  </si>
-  <si>
-    <t>score</t>
-  </si>
-  <si>
-    <t>big</t>
-  </si>
-  <si>
-    <t>ratio</t>
-  </si>
-  <si>
-    <t>price</t>
-  </si>
-  <si>
-    <t>createdAt</t>
-  </si>
-  <si>
-    <t>tags</t>
-  </si>
-  <si>
-    <t>attrs</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t>serverOnly</t>
-  </si>
-  <si>
-    <t>clientOnly</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>int32</t>
-  </si>
-  <si>
-    <t>int64</t>
-  </si>
-  <si>
-    <t>float</t>
-  </si>
-  <si>
-    <t>double</t>
-  </si>
-  <si>
-    <t>datetime</t>
-  </si>
-  <si>
-    <t>array&lt;string&gt;</t>
-  </si>
-  <si>
-    <t>map&lt;string,int&gt;</t>
-  </si>
-  <si>
-    <t>all</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>client</t>
-  </si>
-  <si>
-    <t>server</t>
-  </si>
-  <si>
-    <t>comment</t>
-  </si>
-  <si>
-    <t>srv</t>
-  </si>
-  <si>
-    <t>unique id</t>
+    <t>required label</t>
   </si>
   <si>
     <t>negative int</t>
@@ -110,7 +119,7 @@
     <t>server field</t>
   </si>
   <si>
-    <t>client field</t>
+    <t>unique client field</t>
   </si>
   <si>
     <t>1001</t>
@@ -119,6 +128,9 @@
     <t>Sword</t>
   </si>
   <si>
+    <t>Weapon</t>
+  </si>
+  <si>
     <t>true</t>
   </si>
   <si>
@@ -156,6 +168,9 @@
   </si>
   <si>
     <t>Shield</t>
+  </si>
+  <si>
+    <t>Armor</t>
   </si>
   <si>
     <t>0</t>
@@ -272,13 +287,16 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -305,21 +323,24 @@
         <v>22</v>
       </c>
       <c r="K2" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M2" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
         <v>24</v>
@@ -331,57 +352,60 @@
         <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L3" t="s">
         <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>25</v>
+        <v>29</v>
+      </c>
+      <c r="N3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="J4" t="s">
         <v>9</v>
@@ -390,93 +414,102 @@
         <v>10</v>
       </c>
       <c r="L4" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="M4" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="L5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M5" t="s">
-        <v>49</v>
+        <v>52</v>
+      </c>
+      <c r="N5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="6"/>
     <row r="7">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="L7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="M7" t="s">
-        <v>60</v>
+        <v>64</v>
+      </c>
+      <c r="N7" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -491,83 +524,83 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>